<commit_message>
Finished cleaning up EDM analysis code
</commit_message>
<xml_diff>
--- a/Sheets/BzSim_fitResults.xlsx
+++ b/Sheets/BzSim_fitResults.xlsx
@@ -8,19 +8,30 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{20C2CE32-E635-544D-A81A-D708B7789DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{A128EB77-D23B-A549-B71F-830E0ED7BD00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="1000" windowWidth="27640" windowHeight="16440"/>
+    <workbookView xWindow="960" yWindow="520" windowWidth="10340" windowHeight="16440"/>
   </bookViews>
   <sheets>
     <sheet name="BzSim_fitResults" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
   <si>
     <t>chi2ndf</t>
   </si>
@@ -56,6 +67,12 @@
   </si>
   <si>
     <t>S0S12S18</t>
+  </si>
+  <si>
+    <t>Bz [mrad]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_Bz </t>
   </si>
 </sst>
 </file>
@@ -896,177 +913,208 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E3" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G3" t="s">
         <v>3</v>
       </c>
+      <c r="I3" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C4" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D4" t="s">
         <v>6</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F4" t="s">
         <v>6</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G4" t="s">
         <v>5</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B3">
+      <c r="B5">
         <v>1.23193</v>
       </c>
-      <c r="C3">
+      <c r="C5">
         <v>-3.4237E-3</v>
       </c>
-      <c r="D3">
+      <c r="D5">
         <v>2.0979600000000001E-2</v>
       </c>
-      <c r="E3">
+      <c r="E5">
         <v>0.17380699999999999</v>
       </c>
-      <c r="F3">
+      <c r="F5">
         <v>2.1102099999999999E-2</v>
       </c>
-      <c r="G3">
+      <c r="G5">
         <v>-0.131545</v>
       </c>
-      <c r="H3">
+      <c r="H5">
         <v>1.4914E-2</v>
       </c>
+      <c r="I5">
+        <f>E5/$B$1</f>
+        <v>0.10223941176470588</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
+      <c r="B6">
         <v>1.3388899999999999</v>
       </c>
-      <c r="C4">
+      <c r="C6">
         <v>-3.3000600000000001E-3</v>
       </c>
-      <c r="D4">
+      <c r="D6">
         <v>2.1336299999999999E-2</v>
       </c>
-      <c r="E4">
+      <c r="E6">
         <v>0.15872</v>
       </c>
-      <c r="F4">
+      <c r="F6">
         <v>2.13993E-2</v>
       </c>
-      <c r="G4">
+      <c r="G6">
         <v>-0.39540999999999998</v>
       </c>
-      <c r="H4">
+      <c r="H6">
         <v>1.5144700000000001E-2</v>
       </c>
+      <c r="I6">
+        <f t="shared" ref="I6:I9" si="0">E6/$B$1</f>
+        <v>9.3364705882352947E-2</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B5">
+      <c r="B7">
         <v>1.07422</v>
       </c>
-      <c r="C5">
+      <c r="C7">
         <v>-1.5787900000000001E-3</v>
       </c>
-      <c r="D5">
+      <c r="D7">
         <v>2.1516400000000001E-2</v>
       </c>
-      <c r="E5">
+      <c r="E7">
         <v>0.123597</v>
       </c>
-      <c r="F5">
+      <c r="F7">
         <v>2.1535700000000001E-2</v>
       </c>
-      <c r="G5">
+      <c r="G7">
         <v>-0.34401300000000001</v>
       </c>
-      <c r="H5">
+      <c r="H7">
         <v>1.5252999999999999E-2</v>
       </c>
+      <c r="I7">
+        <f t="shared" si="0"/>
+        <v>7.2704117647058822E-2</v>
+      </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B6">
+      <c r="B8">
         <v>1.1899200000000001</v>
       </c>
-      <c r="C6">
+      <c r="C8">
         <v>-2.3691900000000002E-3</v>
       </c>
-      <c r="D6">
+      <c r="D8">
         <v>1.5151400000000001E-2</v>
       </c>
-      <c r="E6">
+      <c r="E8">
         <v>0.14147199999999999</v>
       </c>
-      <c r="F6">
+      <c r="F8">
         <v>1.51805E-2</v>
       </c>
-      <c r="G6">
+      <c r="G8">
         <v>-0.36990899999999999</v>
       </c>
-      <c r="H6">
+      <c r="H8">
         <v>1.0747700000000001E-2</v>
       </c>
+      <c r="I8">
+        <f t="shared" si="0"/>
+        <v>8.3218823529411762E-2</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>11</v>
       </c>
-      <c r="B7">
+      <c r="B9">
         <v>1.1176900000000001</v>
       </c>
-      <c r="C7">
+      <c r="C9">
         <v>-2.7496299999999999E-3</v>
       </c>
-      <c r="D7">
+      <c r="D9">
         <v>1.22842E-2</v>
       </c>
-      <c r="E7">
+      <c r="E9">
         <v>0.15212999999999999</v>
       </c>
-      <c r="F7">
+      <c r="F9">
         <v>1.2324099999999999E-2</v>
       </c>
-      <c r="G7">
+      <c r="G9">
         <v>-0.28881600000000002</v>
       </c>
-      <c r="H7">
+      <c r="H9">
         <v>8.7201799999999993E-3</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="0"/>
+        <v>8.9488235294117646E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>